<commit_message>
Rewrite paper and audit docs for the F3 revision
Co-authored-by: soloduist-pixiv <soloduist-pixiv@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/2/2016A-mooring/results/results_tables.xlsx
+++ b/2/2016A-mooring/results/results_tables.xlsx
@@ -35,7 +35,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_摘要'!$A$1:$B$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Q1Q2固定球重'!$A$1:$AD$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_Q2调球重'!$A$1:$AE$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_Q2调球重'!$A$1:$AE$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_Q2球重扫描'!$A$1:$AD$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_族对照AB'!$A$1:$AD$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Q3最劣情景'!$A$1:$AE$5</definedName>
@@ -6614,7 +6614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6910,8 +6910,111 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>B_min_mass</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>2220</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>22.05</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>210</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0.985</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>18.5386</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>4.5119</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>15.9969</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>4.4254</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>4.4417</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>4.4582</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>4.4747</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>22.05</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>1644.25</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>1644.25</v>
+      </c>
+      <c r="V3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>1.015</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AE2"/>
+  <autoFilter ref="A1:AE3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>